<commit_message>
Daily NSE scan: 2026-09-25
</commit_message>
<xml_diff>
--- a/output/2026-09-25/enriched_analysis.xlsx
+++ b/output/2026-09-25/enriched_analysis.xlsx
@@ -3669,25 +3669,25 @@
         <v>625.85</v>
       </c>
       <c r="J14" t="n">
-        <v>630.67</v>
+        <v>632.66</v>
       </c>
       <c r="K14" t="n">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
       <c r="L14" t="n">
         <v>64.68000000000001</v>
       </c>
       <c r="M14" t="n">
-        <v>4.7</v>
+        <v>4.44</v>
       </c>
       <c r="N14" t="n">
-        <v>46955184</v>
+        <v>44358875</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>46955184</v>
+        <v>44358875</v>
       </c>
       <c r="Q14" t="n">
         <v>0</v>
@@ -3701,7 +3701,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -3709,7 +3709,7 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.407</v>
+        <v>0.384</v>
       </c>
       <c r="W14" t="n">
         <v>1155</v>
@@ -3751,10 +3751,10 @@
         <v>39.4</v>
       </c>
       <c r="AJ14" t="n">
-        <v>630.668797765033</v>
+        <v>632.6588461812736</v>
       </c>
       <c r="AK14" t="n">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
       <c r="AL14" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>19-06-2026</t>
+          <t>23-06-2026</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -3782,10 +3782,10 @@
         </is>
       </c>
       <c r="AQ14" t="n">
+        <v>90</v>
+      </c>
+      <c r="AR14" t="n">
         <v>94</v>
-      </c>
-      <c r="AR14" t="n">
-        <v>98</v>
       </c>
       <c r="AS14" t="n">
         <v>4</v>
@@ -5021,12 +5021,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -5038,40 +5038,40 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F20" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G20" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="H20" t="n">
         <v>-1</v>
       </c>
       <c r="I20" t="n">
-        <v>177.35</v>
+        <v>216.79</v>
       </c>
       <c r="J20" t="n">
-        <v>169.88</v>
+        <v>210</v>
       </c>
       <c r="K20" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="L20" t="n">
-        <v>61.48</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="M20" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="N20" t="n">
-        <v>5988193</v>
+        <v>5944992</v>
       </c>
       <c r="O20" t="n">
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>5988193</v>
+        <v>5944992</v>
       </c>
       <c r="Q20" t="n">
         <v>0</v>
@@ -5085,124 +5085,124 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.285</v>
+        <v>0.293</v>
       </c>
       <c r="W20" t="n">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="X20" t="n">
-        <v>36.4</v>
+        <v>25.2</v>
       </c>
       <c r="Y20" t="n">
-        <v>-44</v>
+        <v>12</v>
       </c>
       <c r="Z20" t="n">
-        <v>-3.28</v>
+        <v>0.03</v>
       </c>
       <c r="AA20" t="n">
-        <v>141</v>
+        <v>16</v>
       </c>
       <c r="AB20" t="n">
-        <v>-4.05</v>
+        <v>0.03</v>
       </c>
       <c r="AC20" t="n">
-        <v>8.25</v>
+        <v>7.91</v>
       </c>
       <c r="AD20" t="n">
-        <v>0.44</v>
+        <v>-0</v>
       </c>
       <c r="AE20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>-35.96</v>
+        <v>3.16</v>
       </c>
       <c r="AG20" t="n">
-        <v>175.12</v>
+        <v>209.69</v>
       </c>
       <c r="AH20" t="n">
-        <v>179.25</v>
+        <v>196.32</v>
       </c>
       <c r="AI20" t="n">
-        <v>24.8</v>
+        <v>19.5</v>
       </c>
       <c r="AJ20" t="n">
-        <v>169.8778156028369</v>
+        <v>210.0036030944223</v>
       </c>
       <c r="AK20" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM20" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
       <c r="AQ20" t="n">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="AR20" t="n">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="AS20" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AT20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AV20" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="AW20" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="AX20" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="AY20" t="n">
-        <v>2000469</v>
+        <v>0</v>
       </c>
       <c r="AZ20" t="n">
-        <v>5988193</v>
+        <v>1710211</v>
       </c>
       <c r="BA20" t="n">
-        <v>5988193</v>
+        <v>3296491</v>
       </c>
       <c r="BB20" t="n">
-        <v>5988193</v>
+        <v>5944992</v>
       </c>
       <c r="BC20" t="n">
-        <v>5988193</v>
+        <v>5944992</v>
       </c>
       <c r="BD20" t="n">
         <v>0</v>
@@ -5235,10 +5235,10 @@
         <v>0</v>
       </c>
       <c r="BN20" t="n">
-        <v>2000469</v>
+        <v>0</v>
       </c>
       <c r="BO20" t="n">
-        <v>5988193</v>
+        <v>3296491</v>
       </c>
       <c r="BP20" t="n">
         <v>1</v>
@@ -5247,18 +5247,18 @@
         <v>0</v>
       </c>
       <c r="BR20" t="n">
-        <v>0.3341</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -5270,171 +5270,171 @@
         </is>
       </c>
       <c r="E21" t="n">
+        <v>10</v>
+      </c>
+      <c r="F21" t="n">
+        <v>14</v>
+      </c>
+      <c r="G21" t="n">
+        <v>13</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>177.35</v>
+      </c>
+      <c r="J21" t="n">
+        <v>169.88</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L21" t="n">
+        <v>61.48</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N21" t="n">
+        <v>5988193</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" t="n">
+        <v>5988193</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S21" t="b">
+        <v>0</v>
+      </c>
+      <c r="T21" t="n">
+        <v>5</v>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>23-09-2026</t>
+        </is>
+      </c>
+      <c r="V21" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="W21" t="n">
+        <v>210</v>
+      </c>
+      <c r="X21" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="Y21" t="n">
+        <v>-44</v>
+      </c>
+      <c r="Z21" t="n">
+        <v>-3.28</v>
+      </c>
+      <c r="AA21" t="n">
+        <v>141</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>-4.05</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>8.25</v>
+      </c>
+      <c r="AD21" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="AE21" t="b">
         <v>1</v>
       </c>
-      <c r="F21" t="n">
-        <v>18</v>
-      </c>
-      <c r="G21" t="n">
-        <v>17</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>336</v>
-      </c>
-      <c r="J21" t="n">
-        <v>335.41</v>
-      </c>
-      <c r="K21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="L21" t="n">
-        <v>68.48</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="N21" t="n">
-        <v>4081958</v>
-      </c>
-      <c r="O21" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" t="n">
-        <v>4081958</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S21" t="b">
-        <v>0</v>
-      </c>
-      <c r="T21" t="n">
+      <c r="AF21" t="n">
+        <v>-35.96</v>
+      </c>
+      <c r="AG21" t="n">
+        <v>175.12</v>
+      </c>
+      <c r="AH21" t="n">
+        <v>179.25</v>
+      </c>
+      <c r="AI21" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="AJ21" t="n">
+        <v>169.8778156028369</v>
+      </c>
+      <c r="AK21" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="AL21" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AM21" t="inlineStr">
+        <is>
+          <t>Early Accumulation</t>
+        </is>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Early Accumulation</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>16-09-2026</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>23-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ21" t="n">
+        <v>7</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>9</v>
+      </c>
+      <c r="AS21" t="n">
         <v>2</v>
       </c>
-      <c r="U21" t="inlineStr">
-        <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="V21" t="n">
-        <v>0.007</v>
-      </c>
-      <c r="W21" t="n">
-        <v>5507</v>
-      </c>
-      <c r="X21" t="n">
-        <v>9.31</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>43</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>223</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>175</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>6.97</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AE21" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF21" t="n">
-        <v>7</v>
-      </c>
-      <c r="AG21" t="n">
-        <v>365.15</v>
-      </c>
-      <c r="AH21" t="n">
-        <v>335.45</v>
-      </c>
-      <c r="AI21" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="AJ21" t="n">
-        <v>335.4115036976171</v>
-      </c>
-      <c r="AK21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AL21" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AM21" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN21" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO21" t="inlineStr">
-        <is>
-          <t>30-06-2026</t>
-        </is>
-      </c>
-      <c r="AP21" t="inlineStr">
-        <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="AQ21" t="n">
-        <v>49</v>
-      </c>
-      <c r="AR21" t="n">
-        <v>87</v>
-      </c>
-      <c r="AS21" t="n">
-        <v>38</v>
-      </c>
       <c r="AT21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AV21" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AW21" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AX21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AY21" t="n">
-        <v>0</v>
+        <v>2000469</v>
       </c>
       <c r="AZ21" t="n">
-        <v>0</v>
+        <v>5988193</v>
       </c>
       <c r="BA21" t="n">
-        <v>0</v>
+        <v>5988193</v>
       </c>
       <c r="BB21" t="n">
-        <v>1094828</v>
+        <v>5988193</v>
       </c>
       <c r="BC21" t="n">
-        <v>4081958</v>
+        <v>5988193</v>
       </c>
       <c r="BD21" t="n">
         <v>0</v>
@@ -5467,10 +5467,10 @@
         <v>0</v>
       </c>
       <c r="BN21" t="n">
-        <v>0</v>
+        <v>2000469</v>
       </c>
       <c r="BO21" t="n">
-        <v>0</v>
+        <v>5988193</v>
       </c>
       <c r="BP21" t="n">
         <v>1</v>
@@ -5479,18 +5479,18 @@
         <v>0</v>
       </c>
       <c r="BR21" t="n">
-        <v>0</v>
+        <v>0.3341</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -5502,171 +5502,171 @@
         </is>
       </c>
       <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="n">
+        <v>18</v>
+      </c>
+      <c r="G22" t="n">
+        <v>17</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>336</v>
+      </c>
+      <c r="J22" t="n">
+        <v>335.41</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L22" t="n">
+        <v>68.48</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="N22" t="n">
+        <v>4081958</v>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="n">
+        <v>4081958</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S22" t="b">
+        <v>0</v>
+      </c>
+      <c r="T22" t="n">
+        <v>2</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="W22" t="n">
+        <v>5507</v>
+      </c>
+      <c r="X22" t="n">
+        <v>9.31</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>43</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>223</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>175</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>6.97</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="AD22" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="AE22" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="n">
         <v>7</v>
       </c>
-      <c r="F22" t="n">
-        <v>9</v>
-      </c>
-      <c r="G22" t="n">
-        <v>21</v>
-      </c>
-      <c r="H22" t="n">
-        <v>-1</v>
-      </c>
-      <c r="I22" t="n">
-        <v>216.79</v>
-      </c>
-      <c r="J22" t="n">
-        <v>210</v>
-      </c>
-      <c r="K22" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L22" t="n">
-        <v>67.04000000000001</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="N22" t="n">
-        <v>5944992</v>
-      </c>
-      <c r="O22" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" t="n">
-        <v>5944992</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S22" t="b">
-        <v>0</v>
-      </c>
-      <c r="T22" t="n">
-        <v>12</v>
-      </c>
-      <c r="U22" t="inlineStr">
-        <is>
-          <t>17-09-2026</t>
-        </is>
-      </c>
-      <c r="V22" t="n">
-        <v>0.293</v>
-      </c>
-      <c r="W22" t="n">
-        <v>203</v>
-      </c>
-      <c r="X22" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="Y22" t="n">
-        <v>12</v>
-      </c>
-      <c r="Z22" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>16</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="AC22" t="n">
-        <v>7.91</v>
-      </c>
-      <c r="AD22" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AE22" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF22" t="n">
-        <v>3.16</v>
-      </c>
       <c r="AG22" t="n">
-        <v>209.69</v>
+        <v>365.15</v>
       </c>
       <c r="AH22" t="n">
-        <v>196.32</v>
+        <v>335.45</v>
       </c>
       <c r="AI22" t="n">
-        <v>19.5</v>
+        <v>13.5</v>
       </c>
       <c r="AJ22" t="n">
-        <v>210.0036030944223</v>
+        <v>335.4115036976171</v>
       </c>
       <c r="AK22" t="n">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM22" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO22" t="inlineStr">
         <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
           <t>18-08-2026</t>
         </is>
       </c>
-      <c r="AP22" t="inlineStr">
-        <is>
-          <t>17-09-2026</t>
-        </is>
-      </c>
       <c r="AQ22" t="n">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="AR22" t="n">
+        <v>87</v>
+      </c>
+      <c r="AS22" t="n">
         <v>38</v>
       </c>
-      <c r="AS22" t="n">
-        <v>8</v>
-      </c>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV22" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AW22" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="AX22" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="AY22" t="n">
         <v>0</v>
       </c>
       <c r="AZ22" t="n">
-        <v>1710211</v>
+        <v>0</v>
       </c>
       <c r="BA22" t="n">
-        <v>3296491</v>
+        <v>0</v>
       </c>
       <c r="BB22" t="n">
-        <v>5944992</v>
+        <v>1094828</v>
       </c>
       <c r="BC22" t="n">
-        <v>5944992</v>
+        <v>4081958</v>
       </c>
       <c r="BD22" t="n">
         <v>0</v>
@@ -5702,7 +5702,7 @@
         <v>0</v>
       </c>
       <c r="BO22" t="n">
-        <v>3296491</v>
+        <v>0</v>
       </c>
       <c r="BP22" t="n">
         <v>1</v>
@@ -5717,12 +5717,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ENVIRO INFRA ENGINEERS LIMITED</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -5734,40 +5734,40 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
       </c>
       <c r="I23" t="n">
-        <v>201.63</v>
+        <v>230.91</v>
       </c>
       <c r="J23" t="n">
-        <v>191.87</v>
+        <v>234.4</v>
       </c>
       <c r="K23" t="n">
-        <v>5.1</v>
+        <v>-1.5</v>
       </c>
       <c r="L23" t="n">
-        <v>70.02</v>
+        <v>67.13</v>
       </c>
       <c r="M23" t="n">
-        <v>1.34</v>
+        <v>0.3</v>
       </c>
       <c r="N23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="Q23" t="n">
         <v>0</v>
@@ -5785,96 +5785,96 @@
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="V23" t="n">
-        <v>0.038</v>
+        <v>0.043</v>
       </c>
       <c r="W23" t="n">
-        <v>3539</v>
+        <v>693</v>
       </c>
       <c r="X23" t="n">
-        <v>21</v>
+        <v>11.3</v>
       </c>
       <c r="Y23" t="n">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="Z23" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="AA23" t="n">
-        <v>-9</v>
+        <v>1</v>
       </c>
       <c r="AB23" t="n">
-        <v>2.04</v>
+        <v>6.54</v>
       </c>
       <c r="AC23" t="n">
-        <v>20.8</v>
+        <v>14.8</v>
       </c>
       <c r="AD23" t="n">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="AE23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="AG23" t="n">
-        <v>207.06</v>
+        <v>227.44</v>
       </c>
       <c r="AH23" t="n">
-        <v>193.72</v>
+        <v>205</v>
       </c>
       <c r="AI23" t="n">
-        <v>36.4</v>
+        <v>37.8</v>
       </c>
       <c r="AJ23" t="n">
-        <v>191.8684857142857</v>
+        <v>234.4008293560754</v>
       </c>
       <c r="AK23" t="n">
-        <v>5.1</v>
+        <v>-1.5</v>
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM23" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO23" t="inlineStr">
         <is>
-          <t>31-08-2026</t>
+          <t>21-09-2026</t>
         </is>
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="AQ23" t="n">
         <v>2</v>
       </c>
       <c r="AR23" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="AS23" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="AT23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AU23" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV23" t="n">
         <v>3</v>
@@ -5886,19 +5886,19 @@
         <v>3</v>
       </c>
       <c r="AY23" t="n">
-        <v>0</v>
+        <v>2995877</v>
       </c>
       <c r="AZ23" t="n">
-        <v>0</v>
+        <v>2995877</v>
       </c>
       <c r="BA23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="BB23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="BC23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="BD23" t="n">
         <v>0</v>
@@ -5931,30 +5931,30 @@
         <v>0</v>
       </c>
       <c r="BN23" t="n">
-        <v>0</v>
+        <v>2995877</v>
       </c>
       <c r="BO23" t="n">
-        <v>13430794</v>
+        <v>2995877</v>
       </c>
       <c r="BP23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ23" t="n">
         <v>0</v>
       </c>
       <c r="BR23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -5966,40 +5966,40 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G24" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>646.6</v>
+        <v>249.6</v>
       </c>
       <c r="J24" t="n">
-        <v>593.62</v>
+        <v>243.52</v>
       </c>
       <c r="K24" t="n">
-        <v>8.9</v>
+        <v>2.5</v>
       </c>
       <c r="L24" t="n">
-        <v>74.02</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="M24" t="n">
-        <v>0.25</v>
+        <v>1.11</v>
       </c>
       <c r="N24" t="n">
-        <v>2458195</v>
+        <v>11080000</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
       </c>
       <c r="P24" t="n">
-        <v>2458195</v>
+        <v>11080000</v>
       </c>
       <c r="Q24" t="n">
         <v>0</v>
@@ -6017,118 +6017,120 @@
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.024</v>
+        <v>0.165</v>
       </c>
       <c r="W24" t="n">
-        <v>1005</v>
-      </c>
-      <c r="X24" t="inlineStr"/>
+        <v>671</v>
+      </c>
+      <c r="X24" t="n">
+        <v>56.1</v>
+      </c>
       <c r="Y24" t="n">
-        <v>-2</v>
+        <v>3</v>
       </c>
       <c r="Z24" t="n">
-        <v>5</v>
+        <v>2.99</v>
       </c>
       <c r="AA24" t="n">
-        <v>-152</v>
+        <v>97</v>
       </c>
       <c r="AB24" t="n">
-        <v>-6.5</v>
+        <v>1</v>
       </c>
       <c r="AC24" t="n">
-        <v>9.24</v>
+        <v>11.6</v>
       </c>
       <c r="AD24" t="n">
-        <v>2.23</v>
+        <v>0</v>
       </c>
       <c r="AE24" t="b">
         <v>1</v>
       </c>
       <c r="AF24" t="n">
-        <v>6</v>
+        <v>16.21</v>
       </c>
       <c r="AG24" t="n">
-        <v>594.08</v>
+        <v>255.85</v>
       </c>
       <c r="AH24" t="n">
-        <v>547.55</v>
+        <v>187.89</v>
       </c>
       <c r="AI24" t="n">
-        <v>29.2</v>
+        <v>95</v>
       </c>
       <c r="AJ24" t="n">
-        <v>593.6235208886742</v>
+        <v>238.0921052631579</v>
       </c>
       <c r="AK24" t="n">
-        <v>8.9</v>
+        <v>4.8</v>
       </c>
       <c r="AL24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO24" t="inlineStr">
         <is>
-          <t>28-08-2026</t>
+          <t>06-08-2026</t>
         </is>
       </c>
       <c r="AP24" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="AQ24" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="AR24" t="n">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="AS24" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="AT24" t="n">
         <v>0</v>
       </c>
       <c r="AU24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV24" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AW24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AX24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AY24" t="n">
         <v>0</v>
       </c>
       <c r="AZ24" t="n">
-        <v>322003</v>
+        <v>0</v>
       </c>
       <c r="BA24" t="n">
-        <v>2458195</v>
+        <v>0</v>
       </c>
       <c r="BB24" t="n">
-        <v>2458195</v>
+        <v>18095000</v>
       </c>
       <c r="BC24" t="n">
-        <v>2458195</v>
+        <v>18095000</v>
       </c>
       <c r="BD24" t="n">
         <v>0</v>
@@ -6164,10 +6166,10 @@
         <v>0</v>
       </c>
       <c r="BO24" t="n">
-        <v>2458195</v>
+        <v>0</v>
       </c>
       <c r="BP24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="BQ24" t="n">
         <v>0</v>
@@ -6179,12 +6181,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>ENVIRO INFRA ENGINEERS LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -6196,40 +6198,40 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F25" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="G25" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>249.6</v>
+        <v>201.63</v>
       </c>
       <c r="J25" t="n">
-        <v>243.52</v>
+        <v>191.87</v>
       </c>
       <c r="K25" t="n">
-        <v>2.5</v>
+        <v>5.1</v>
       </c>
       <c r="L25" t="n">
-        <v>67.65000000000001</v>
+        <v>70.02</v>
       </c>
       <c r="M25" t="n">
-        <v>1.11</v>
+        <v>1.34</v>
       </c>
       <c r="N25" t="n">
-        <v>11080000</v>
+        <v>13430794</v>
       </c>
       <c r="O25" t="n">
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>11080000</v>
+        <v>13430794</v>
       </c>
       <c r="Q25" t="n">
         <v>0</v>
@@ -6247,105 +6249,105 @@
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.165</v>
+        <v>0.038</v>
       </c>
       <c r="W25" t="n">
-        <v>671</v>
+        <v>3539</v>
       </c>
       <c r="X25" t="n">
-        <v>56.1</v>
+        <v>21</v>
       </c>
       <c r="Y25" t="n">
+        <v>-4</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>51</v>
+      </c>
+      <c r="AA25" t="n">
+        <v>-9</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="AD25" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="AE25" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>21</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>207.06</v>
+      </c>
+      <c r="AH25" t="n">
+        <v>193.72</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>36.4</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>191.8684857142857</v>
+      </c>
+      <c r="AK25" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>31-08-2026</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>02-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>25</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>23</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
         <v>3</v>
       </c>
-      <c r="Z25" t="n">
-        <v>2.99</v>
-      </c>
-      <c r="AA25" t="n">
-        <v>97</v>
-      </c>
-      <c r="AB25" t="n">
-        <v>1</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="AD25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE25" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF25" t="n">
-        <v>16.21</v>
-      </c>
-      <c r="AG25" t="n">
-        <v>255.85</v>
-      </c>
-      <c r="AH25" t="n">
-        <v>187.89</v>
-      </c>
-      <c r="AI25" t="n">
-        <v>95</v>
-      </c>
-      <c r="AJ25" t="n">
-        <v>238.0921052631579</v>
-      </c>
-      <c r="AK25" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AM25" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN25" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO25" t="inlineStr">
-        <is>
-          <t>06-08-2026</t>
-        </is>
-      </c>
-      <c r="AP25" t="inlineStr">
-        <is>
-          <t>25-08-2026</t>
-        </is>
-      </c>
-      <c r="AQ25" t="n">
-        <v>19</v>
-      </c>
-      <c r="AR25" t="n">
-        <v>50</v>
-      </c>
-      <c r="AS25" t="n">
-        <v>31</v>
-      </c>
-      <c r="AT25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU25" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV25" t="n">
-        <v>0</v>
-      </c>
       <c r="AW25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AX25" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AY25" t="n">
         <v>0</v>
@@ -6354,13 +6356,13 @@
         <v>0</v>
       </c>
       <c r="BA25" t="n">
-        <v>0</v>
+        <v>13430794</v>
       </c>
       <c r="BB25" t="n">
-        <v>18095000</v>
+        <v>13430794</v>
       </c>
       <c r="BC25" t="n">
-        <v>18095000</v>
+        <v>13430794</v>
       </c>
       <c r="BD25" t="n">
         <v>0</v>
@@ -6396,7 +6398,7 @@
         <v>0</v>
       </c>
       <c r="BO25" t="n">
-        <v>0</v>
+        <v>13430794</v>
       </c>
       <c r="BP25" t="n">
         <v>2</v>
@@ -6411,12 +6413,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -6428,40 +6430,40 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F26" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>230.91</v>
+        <v>646.6</v>
       </c>
       <c r="J26" t="n">
-        <v>234.4</v>
+        <v>593.62</v>
       </c>
       <c r="K26" t="n">
-        <v>-1.5</v>
+        <v>8.9</v>
       </c>
       <c r="L26" t="n">
-        <v>67.13</v>
+        <v>74.02</v>
       </c>
       <c r="M26" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="N26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="O26" t="n">
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="Q26" t="n">
         <v>0</v>
@@ -6479,96 +6481,94 @@
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.043</v>
+        <v>0.024</v>
       </c>
       <c r="W26" t="n">
-        <v>693</v>
-      </c>
-      <c r="X26" t="n">
-        <v>11.3</v>
-      </c>
+        <v>1005</v>
+      </c>
+      <c r="X26" t="inlineStr"/>
       <c r="Y26" t="n">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="Z26" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="AA26" t="n">
-        <v>1</v>
+        <v>-152</v>
       </c>
       <c r="AB26" t="n">
-        <v>6.54</v>
+        <v>-6.5</v>
       </c>
       <c r="AC26" t="n">
-        <v>14.8</v>
+        <v>9.24</v>
       </c>
       <c r="AD26" t="n">
-        <v>0.11</v>
+        <v>2.23</v>
       </c>
       <c r="AE26" t="b">
         <v>1</v>
       </c>
       <c r="AF26" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AG26" t="n">
-        <v>227.44</v>
+        <v>594.08</v>
       </c>
       <c r="AH26" t="n">
-        <v>205</v>
+        <v>547.55</v>
       </c>
       <c r="AI26" t="n">
-        <v>37.8</v>
+        <v>29.2</v>
       </c>
       <c r="AJ26" t="n">
-        <v>234.4008293560754</v>
+        <v>593.6235208886742</v>
       </c>
       <c r="AK26" t="n">
-        <v>-1.5</v>
+        <v>8.9</v>
       </c>
       <c r="AL26" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM26" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO26" t="inlineStr">
         <is>
-          <t>21-09-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="AP26" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
       <c r="AQ26" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="AR26" t="n">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="AS26" t="n">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="AT26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AU26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AV26" t="n">
         <v>3</v>
@@ -6580,19 +6580,19 @@
         <v>3</v>
       </c>
       <c r="AY26" t="n">
-        <v>2995877</v>
+        <v>0</v>
       </c>
       <c r="AZ26" t="n">
-        <v>2995877</v>
+        <v>322003</v>
       </c>
       <c r="BA26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="BB26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="BC26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="BD26" t="n">
         <v>0</v>
@@ -6625,19 +6625,19 @@
         <v>0</v>
       </c>
       <c r="BN26" t="n">
-        <v>2995877</v>
+        <v>0</v>
       </c>
       <c r="BO26" t="n">
-        <v>2995877</v>
+        <v>2458195</v>
       </c>
       <c r="BP26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ26" t="n">
         <v>0</v>
       </c>
       <c r="BR26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -6875,12 +6875,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NUPUR RECYCLERS LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -6892,40 +6892,40 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F28" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G28" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H28" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>165</v>
+        <v>147.51</v>
       </c>
       <c r="J28" t="n">
-        <v>83.06</v>
+        <v>171.84</v>
       </c>
       <c r="K28" t="n">
-        <v>98.7</v>
+        <v>-14.2</v>
       </c>
       <c r="L28" t="n">
-        <v>72.53</v>
+        <v>74.59</v>
       </c>
       <c r="M28" t="n">
-        <v>0.42</v>
+        <v>1.1</v>
       </c>
       <c r="N28" t="n">
-        <v>4186225</v>
+        <v>10997624</v>
       </c>
       <c r="O28" t="n">
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>4186225</v>
+        <v>10997624</v>
       </c>
       <c r="Q28" t="n">
         <v>0</v>
@@ -6939,94 +6939,94 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.037</v>
+        <v>0.059</v>
       </c>
       <c r="W28" t="n">
-        <v>1140</v>
+        <v>1871</v>
       </c>
       <c r="X28" t="n">
-        <v>122</v>
+        <v>42.9</v>
       </c>
       <c r="Y28" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Z28" t="n">
-        <v>1.43</v>
+        <v>17</v>
       </c>
       <c r="AA28" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="AB28" t="n">
-        <v>0.34</v>
+        <v>0.8</v>
       </c>
       <c r="AC28" t="n">
-        <v>9.710000000000001</v>
+        <v>30.3</v>
       </c>
       <c r="AD28" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AE28" t="b">
         <v>1</v>
       </c>
       <c r="AF28" t="n">
-        <v>3.67</v>
+        <v>23</v>
       </c>
       <c r="AG28" t="n">
-        <v>121.61</v>
+        <v>182.53</v>
       </c>
       <c r="AH28" t="n">
-        <v>75.76000000000001</v>
+        <v>499.2</v>
       </c>
       <c r="AI28" t="n">
-        <v>229.7</v>
+        <v>19.9</v>
       </c>
       <c r="AJ28" t="n">
-        <v>83.06001984126983</v>
+        <v>170.7900804020101</v>
       </c>
       <c r="AK28" t="n">
-        <v>98.7</v>
+        <v>-13.6</v>
       </c>
       <c r="AL28" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM28" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN28" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
       <c r="AP28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
       <c r="AQ28" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="AR28" t="n">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="AS28" t="n">
-        <v>93</v>
+        <v>16</v>
       </c>
       <c r="AT28" t="n">
         <v>0</v>
@@ -7035,13 +7035,13 @@
         <v>0</v>
       </c>
       <c r="AV28" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AW28" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AX28" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="AY28" t="n">
         <v>0</v>
@@ -7050,13 +7050,13 @@
         <v>0</v>
       </c>
       <c r="BA28" t="n">
-        <v>0</v>
+        <v>28919876</v>
       </c>
       <c r="BB28" t="n">
-        <v>0</v>
+        <v>33987226</v>
       </c>
       <c r="BC28" t="n">
-        <v>0</v>
+        <v>33987226</v>
       </c>
       <c r="BD28" t="n">
         <v>0</v>
@@ -7092,7 +7092,7 @@
         <v>0</v>
       </c>
       <c r="BO28" t="n">
-        <v>0</v>
+        <v>28919876</v>
       </c>
       <c r="BP28" t="n">
         <v>1</v>
@@ -7107,12 +7107,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>NUPUR RECYCLERS LIMITED</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -7124,40 +7124,40 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G29" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I29" t="n">
-        <v>147.51</v>
+        <v>165</v>
       </c>
       <c r="J29" t="n">
-        <v>171.84</v>
+        <v>83.06</v>
       </c>
       <c r="K29" t="n">
-        <v>-14.2</v>
+        <v>98.7</v>
       </c>
       <c r="L29" t="n">
-        <v>74.59</v>
+        <v>72.53</v>
       </c>
       <c r="M29" t="n">
-        <v>1.1</v>
+        <v>0.42</v>
       </c>
       <c r="N29" t="n">
-        <v>10997624</v>
+        <v>4186225</v>
       </c>
       <c r="O29" t="n">
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>10997624</v>
+        <v>4186225</v>
       </c>
       <c r="Q29" t="n">
         <v>0</v>
@@ -7171,94 +7171,94 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.059</v>
+        <v>0.037</v>
       </c>
       <c r="W29" t="n">
-        <v>1871</v>
+        <v>1140</v>
       </c>
       <c r="X29" t="n">
-        <v>42.9</v>
+        <v>122</v>
       </c>
       <c r="Y29" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="Z29" t="n">
-        <v>17</v>
+        <v>1.43</v>
       </c>
       <c r="AA29" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="AB29" t="n">
-        <v>0.8</v>
+        <v>0.34</v>
       </c>
       <c r="AC29" t="n">
-        <v>30.3</v>
+        <v>9.710000000000001</v>
       </c>
       <c r="AD29" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="AE29" t="b">
         <v>1</v>
       </c>
       <c r="AF29" t="n">
-        <v>23</v>
+        <v>3.67</v>
       </c>
       <c r="AG29" t="n">
-        <v>182.53</v>
+        <v>121.61</v>
       </c>
       <c r="AH29" t="n">
-        <v>499.2</v>
+        <v>75.76000000000001</v>
       </c>
       <c r="AI29" t="n">
-        <v>19.9</v>
+        <v>229.7</v>
       </c>
       <c r="AJ29" t="n">
-        <v>170.7900804020101</v>
+        <v>83.06001984126983</v>
       </c>
       <c r="AK29" t="n">
-        <v>-13.6</v>
+        <v>98.7</v>
       </c>
       <c r="AL29" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="AM29" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Stale Accumulation</t>
         </is>
       </c>
       <c r="AN29" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO29" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AP29" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AQ29" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="AR29" t="n">
-        <v>31</v>
+        <v>93</v>
       </c>
       <c r="AS29" t="n">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="AT29" t="n">
         <v>0</v>
@@ -7267,13 +7267,13 @@
         <v>0</v>
       </c>
       <c r="AV29" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="AW29" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AX29" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AY29" t="n">
         <v>0</v>
@@ -7282,13 +7282,13 @@
         <v>0</v>
       </c>
       <c r="BA29" t="n">
-        <v>28919876</v>
+        <v>0</v>
       </c>
       <c r="BB29" t="n">
-        <v>33987226</v>
+        <v>0</v>
       </c>
       <c r="BC29" t="n">
-        <v>33987226</v>
+        <v>0</v>
       </c>
       <c r="BD29" t="n">
         <v>0</v>
@@ -7324,7 +7324,7 @@
         <v>0</v>
       </c>
       <c r="BO29" t="n">
-        <v>28919876</v>
+        <v>0</v>
       </c>
       <c r="BP29" t="n">
         <v>1</v>
@@ -9911,25 +9911,25 @@
         <v>26.36</v>
       </c>
       <c r="J41" t="n">
-        <v>32.21</v>
+        <v>31.66</v>
       </c>
       <c r="K41" t="n">
-        <v>-18.2</v>
+        <v>-16.7</v>
       </c>
       <c r="L41" t="n">
         <v>61.81</v>
       </c>
       <c r="M41" t="n">
-        <v>0.83</v>
+        <v>0.76</v>
       </c>
       <c r="N41" t="n">
-        <v>8341370</v>
+        <v>7567370</v>
       </c>
       <c r="O41" t="n">
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>8341370</v>
+        <v>7567370</v>
       </c>
       <c r="Q41" t="n">
         <v>0</v>
@@ -9943,7 +9943,7 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
@@ -9951,7 +9951,7 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0.299</v>
+        <v>0.271</v>
       </c>
       <c r="W41" t="n">
         <v>279</v>
@@ -9993,10 +9993,10 @@
         <v>5.1</v>
       </c>
       <c r="AJ41" t="n">
-        <v>32.20606177606177</v>
+        <v>31.6626359832636</v>
       </c>
       <c r="AK41" t="n">
-        <v>-18.2</v>
+        <v>-16.7</v>
       </c>
       <c r="AL41" t="inlineStr">
         <is>
@@ -10015,7 +10015,7 @@
       </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="AP41" t="inlineStr">
@@ -10024,10 +10024,10 @@
         </is>
       </c>
       <c r="AQ41" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="AR41" t="n">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="AS41" t="n">
         <v>2</v>
@@ -11763,28 +11763,28 @@
         <v>806.1</v>
       </c>
       <c r="J49" t="n">
-        <v>241.63</v>
+        <v>243.4</v>
       </c>
       <c r="K49" t="n">
-        <v>233.6</v>
+        <v>231.2</v>
       </c>
       <c r="L49" t="n">
         <v>60.24</v>
       </c>
       <c r="M49" t="n">
-        <v>7.67</v>
+        <v>3.65</v>
       </c>
       <c r="N49" t="n">
-        <v>76695745</v>
+        <v>36537959</v>
       </c>
       <c r="O49" t="n">
-        <v>80376270</v>
+        <v>40279632</v>
       </c>
       <c r="P49" t="n">
-        <v>-3680525</v>
+        <v>-3741673</v>
       </c>
       <c r="Q49" t="n">
-        <v>104.8</v>
+        <v>110.24</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -11795,7 +11795,7 @@
         <v>1</v>
       </c>
       <c r="T49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
@@ -11845,10 +11845,10 @@
         <v>285.8</v>
       </c>
       <c r="AJ49" t="n">
-        <v>241.6253276457393</v>
+        <v>243.3981654187428</v>
       </c>
       <c r="AK49" t="n">
-        <v>233.6</v>
+        <v>231.2</v>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
@@ -11867,7 +11867,7 @@
       </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>23-06-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
@@ -11876,10 +11876,10 @@
         </is>
       </c>
       <c r="AQ49" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AR49" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="AS49" t="n">
         <v>92</v>
@@ -13395,19 +13395,19 @@
         <v>625.85</v>
       </c>
       <c r="D14" t="n">
-        <v>630.67</v>
+        <v>632.66</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
       <c r="F14" t="n">
         <v>64.68000000000001</v>
       </c>
       <c r="G14" t="n">
-        <v>4.7</v>
+        <v>4.44</v>
       </c>
       <c r="H14" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -13593,245 +13593,245 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AFFORDABLE</t>
+          <t>TAINWALCHM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
+          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>177.35</v>
+        <v>216.79</v>
       </c>
       <c r="D20" t="n">
-        <v>169.88</v>
+        <v>210</v>
       </c>
       <c r="E20" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="F20" t="n">
-        <v>61.48</v>
+        <v>67.04000000000001</v>
       </c>
       <c r="G20" t="n">
-        <v>0.6</v>
+        <v>0.59</v>
       </c>
       <c r="H20" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>17-09-2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>AFFORDABLE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>AFFORDABLE ROBOTIC &amp; AUTOMATION LIMITED</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>336</v>
+        <v>177.35</v>
       </c>
       <c r="D21" t="n">
-        <v>335.41</v>
+        <v>169.88</v>
       </c>
       <c r="E21" t="n">
-        <v>0.2</v>
+        <v>4.4</v>
       </c>
       <c r="F21" t="n">
-        <v>68.48</v>
+        <v>61.48</v>
       </c>
       <c r="G21" t="n">
-        <v>0.41</v>
+        <v>0.6</v>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TAINWALCHM</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TAINWALA CHEMICALS AND PLASTICS (INDIA) LIMITED</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>216.79</v>
+        <v>336</v>
       </c>
       <c r="D22" t="n">
-        <v>210</v>
+        <v>335.41</v>
       </c>
       <c r="E22" t="n">
-        <v>3.2</v>
+        <v>0.2</v>
       </c>
       <c r="F22" t="n">
-        <v>67.04000000000001</v>
+        <v>68.48</v>
       </c>
       <c r="G22" t="n">
-        <v>0.59</v>
+        <v>0.41</v>
       </c>
       <c r="H22" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>17-09-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>EIEL</t>
+          <t>JAYAGROGN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ENVIRO INFRA ENGINEERS LIMITED</t>
+          <t>Jayant Agro-Organics Limited</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>201.63</v>
+        <v>230.91</v>
       </c>
       <c r="D23" t="n">
-        <v>191.87</v>
+        <v>234.4</v>
       </c>
       <c r="E23" t="n">
-        <v>5.1</v>
+        <v>-1.5</v>
       </c>
       <c r="F23" t="n">
-        <v>70.02</v>
+        <v>67.13</v>
       </c>
       <c r="G23" t="n">
-        <v>1.34</v>
+        <v>0.3</v>
       </c>
       <c r="H23" t="n">
         <v>3</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>02-09-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>CHEMBONDCH</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>CHEMBOND CHEMICALS LIMITED</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>646.6</v>
+        <v>249.6</v>
       </c>
       <c r="D24" t="n">
-        <v>593.62</v>
+        <v>243.52</v>
       </c>
       <c r="E24" t="n">
-        <v>8.9</v>
+        <v>2.5</v>
       </c>
       <c r="F24" t="n">
-        <v>74.02</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="G24" t="n">
-        <v>0.25</v>
+        <v>1.11</v>
       </c>
       <c r="H24" t="n">
         <v>3</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>11-09-2026</t>
+          <t>25-08-2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CHEMBONDCH</t>
+          <t>EIEL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CHEMBOND CHEMICALS LIMITED</t>
+          <t>ENVIRO INFRA ENGINEERS LIMITED</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>249.6</v>
+        <v>201.63</v>
       </c>
       <c r="D25" t="n">
-        <v>243.52</v>
+        <v>191.87</v>
       </c>
       <c r="E25" t="n">
-        <v>2.5</v>
+        <v>5.1</v>
       </c>
       <c r="F25" t="n">
-        <v>67.65000000000001</v>
+        <v>70.02</v>
       </c>
       <c r="G25" t="n">
-        <v>1.11</v>
+        <v>1.34</v>
       </c>
       <c r="H25" t="n">
         <v>3</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>25-08-2026</t>
+          <t>02-09-2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>JAYAGROGN</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jayant Agro-Organics Limited</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>230.91</v>
+        <v>646.6</v>
       </c>
       <c r="D26" t="n">
-        <v>234.4</v>
+        <v>593.62</v>
       </c>
       <c r="E26" t="n">
-        <v>-1.5</v>
+        <v>8.9</v>
       </c>
       <c r="F26" t="n">
-        <v>67.13</v>
+        <v>74.02</v>
       </c>
       <c r="G26" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="H26" t="n">
         <v>3</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>11-09-2026</t>
         </is>
       </c>
     </row>
@@ -13873,70 +13873,70 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NRL</t>
+          <t>SILVERTUC</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>NUPUR RECYCLERS LIMITED</t>
+          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>165</v>
+        <v>147.51</v>
       </c>
       <c r="D28" t="n">
-        <v>83.06</v>
+        <v>171.84</v>
       </c>
       <c r="E28" t="n">
-        <v>98.7</v>
+        <v>-14.2</v>
       </c>
       <c r="F28" t="n">
-        <v>72.53</v>
+        <v>74.59</v>
       </c>
       <c r="G28" t="n">
-        <v>0.42</v>
+        <v>1.1</v>
       </c>
       <c r="H28" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>24-06-2026</t>
+          <t>09-09-2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SILVERTUC</t>
+          <t>NRL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SILVER TOUCH TECHNOLOGIES LIMITED</t>
+          <t>NUPUR RECYCLERS LIMITED</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>147.51</v>
+        <v>165</v>
       </c>
       <c r="D29" t="n">
-        <v>171.84</v>
+        <v>83.06</v>
       </c>
       <c r="E29" t="n">
-        <v>-14.2</v>
+        <v>98.7</v>
       </c>
       <c r="F29" t="n">
-        <v>74.59</v>
+        <v>72.53</v>
       </c>
       <c r="G29" t="n">
-        <v>1.1</v>
+        <v>0.42</v>
       </c>
       <c r="H29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>09-09-2026</t>
+          <t>24-06-2026</t>
         </is>
       </c>
     </row>
@@ -14340,19 +14340,19 @@
         <v>26.36</v>
       </c>
       <c r="D41" t="n">
-        <v>32.21</v>
+        <v>31.66</v>
       </c>
       <c r="E41" t="n">
-        <v>-18.2</v>
+        <v>-16.7</v>
       </c>
       <c r="F41" t="n">
         <v>61.81</v>
       </c>
       <c r="G41" t="n">
-        <v>0.83</v>
+        <v>0.76</v>
       </c>
       <c r="H41" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -14620,19 +14620,19 @@
         <v>806.1</v>
       </c>
       <c r="D49" t="n">
-        <v>241.63</v>
+        <v>243.4</v>
       </c>
       <c r="E49" t="n">
-        <v>233.6</v>
+        <v>231.2</v>
       </c>
       <c r="F49" t="n">
         <v>60.24</v>
       </c>
       <c r="G49" t="n">
-        <v>7.67</v>
+        <v>3.65</v>
       </c>
       <c r="H49" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>

</xml_diff>